<commit_message>
data(GEM2026Q1): collect 8610.HK BBSB International with independent review
Replace the empty official-source-only shell with the real cohort.
- Prospectus (69 fields), allotment (18) and GEM extension (15) payloads were
  extracted from the HKEX prospectus and allotment results announcement, validated
  with 0 errors, and independently reviewed field by field against the original
  pages by a separate reviewer (reports name the payload sha256).
- Year-1 is the 6M period ended 2025-06-30 from the audited Track Record
  (annualised x2 for sales, profit before tax and profit for the period; BC=0.5).
- Canonical layout mirrors GEM2025Q4: workbook in cohorts/, payloads and audits in
  out/gem_2026q1/, config paths repointed, export and codebook regenerated.
- audit: 69/69 prospectus, 18/18 allot, 15/15 GEM cells matched; cross-check
  0 errors. Ten GEM extension fields stay NA/NaN because the prospectus does not
  disclose them.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/cohorts/HKIPO-GEM2026Q1.xlsx
+++ b/pipeline/cohorts/HKIPO-GEM2026Q1.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="0000"/>
@@ -30,9 +30,11 @@
     <numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
     <numFmt numFmtId="170" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="173" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +84,14 @@
       <b val="1"/>
       <color theme="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -199,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -321,6 +331,37 @@
     </xf>
     <xf numFmtId="170" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1971,6 +2012,9 @@
       <c r="D2" t="n">
         <v>0.6</v>
       </c>
+      <c r="E2" t="n">
+        <v>10745.13</v>
+      </c>
       <c r="F2" t="n">
         <v>75000000</v>
       </c>
@@ -1980,6 +2024,21 @@
       <c r="H2" t="n">
         <v>300000000</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Civil engineering contractor in Malaysia specialising in bridge engineering services as a subcontractor for large-scale transportation infrastructure engineering projects</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Cayman Islands</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Listing on GEM of the Stock Exchange by way of Share Offer (Public Offer and Placing)</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>Lego Corporate Finance Limited</t>
@@ -1988,10 +2047,529 @@
       <c r="M2" t="inlineStr">
         <is>
           <t>BDO Limited</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="O2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="P2" t="n">
+        <v>375000000</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>375000000</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="T2" t="n">
+        <v>112500000</v>
+      </c>
+      <c r="U2" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>MYR</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>113572000</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>109044000</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>114046000</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>63611000</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>53800000</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>57001000</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>49961000</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>55244000</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>57045000</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>76757000</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>133002000</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>147972000</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>-13098000</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>33273000</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>11886000</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>-14460000</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>26189000</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>6402000</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="AU2" t="n">
         <v>1</v>
+      </c>
+      <c r="AV2" s="34" t="n">
+        <v>46022</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>-0.07692300000000001</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0.153846</v>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>At low</t>
+        </is>
+      </c>
+      <c r="BC2" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="BE2" s="42" t="n">
+        <v>45838</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>-3480000</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>9086000</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="BR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>Family (Datuk Tan and spouse Datin Pan, via BBSB Overseas)</t>
+        </is>
+      </c>
+      <c r="BW2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>6042000</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>GEM</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="CC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>602030</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>HSICS (Hang Seng Industry Classification System) 2026</t>
+        </is>
+      </c>
+      <c r="CF2" s="42" t="n">
+        <v>45807</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="CH2" t="inlineStr">
+        <is>
+          <t>Petaling Jaya, Malaysia</t>
+        </is>
+      </c>
+      <c r="CJ2" t="inlineStr">
+        <is>
+          <t>IFRS Accounting Standards</t>
+        </is>
+      </c>
+      <c r="CK2" s="42" t="n">
+        <v>44927</v>
+      </c>
+      <c r="CL2" s="42" t="n">
+        <v>45291</v>
+      </c>
+      <c r="CM2" s="42" t="n">
+        <v>45292</v>
+      </c>
+      <c r="CN2" s="42" t="n">
+        <v>45657</v>
+      </c>
+      <c r="CO2" s="42" t="n">
+        <v>45658</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>73986000</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>5943000</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>3201000</v>
+      </c>
+      <c r="CS2" s="42" t="n">
+        <v>46022</v>
+      </c>
+      <c r="CT2" s="42" t="n">
+        <v>46030</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>15806000</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>113000</v>
+      </c>
+      <c r="CX2" t="inlineStr">
+        <is>
+          <t>Unqualified opinion</t>
+        </is>
+      </c>
+      <c r="CY2" t="n">
+        <v>25300000</v>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>Mr. Choy Joo Seong; Mr. Tan Nam Joo</t>
+        </is>
+      </c>
+      <c r="DA2" t="n">
+        <v>0.186624</v>
+      </c>
+      <c r="DB2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="DC2" t="n">
+        <v>145089</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>134314148000</v>
+      </c>
+      <c r="DE2" t="inlineStr">
+        <is>
+          <t>Subscription level 10,745.13 times</t>
+        </is>
+      </c>
+      <c r="DF2" s="42" t="n">
+        <v>46031</v>
+      </c>
+      <c r="DG2" s="42" t="n">
+        <v>46034</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>112500000</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM2" t="inlineStr">
+        <is>
+          <t>No clawback: Claw-back triggered No; re-allocation procedure not applied; final Public Offer 12,500,000 and Placing 112,500,000 Shares</t>
+        </is>
+      </c>
+      <c r="DN2" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="DO2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="DP2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="DQ2" t="n">
+        <v>0.2033</v>
+      </c>
+      <c r="DR2" t="inlineStr">
+        <is>
+          <t>Free float denominator = total issued shares upon listing (col_CZ); numerator = offer shares minus cornerstone allocation</t>
+        </is>
+      </c>
+      <c r="DS2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="DT2" t="n">
+        <v>-0.00016594</v>
+      </c>
+      <c r="DU2" t="n">
+        <v>1</v>
+      </c>
+      <c r="DV2" t="n">
+        <v>0.0321107</v>
+      </c>
+      <c r="DW2" t="n">
+        <v>53950000000</v>
+      </c>
+      <c r="DX2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="DY2" t="n">
+        <v>0.116667</v>
+      </c>
+      <c r="DZ2" t="n">
+        <v>8750000</v>
+      </c>
+      <c r="EA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="EB2" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="EC2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="ED2" t="n">
+        <v>120963660</v>
+      </c>
+      <c r="EE2" t="n">
+        <v>0.967709</v>
+      </c>
+      <c r="EI2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="EJ2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="EK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="EL2" t="n">
+        <v>0.116667</v>
+      </c>
+      <c r="EM2" t="n">
+        <v>0.006655</v>
+      </c>
+      <c r="EN2" t="n">
+        <v>-0.07703699999999999</v>
+      </c>
+      <c r="EO2" t="n">
+        <v>0.9933999999999999</v>
+      </c>
+      <c r="EP2" t="n">
+        <v>1.0835</v>
+      </c>
+      <c r="EQ2" t="n">
+        <v>11622003.5</v>
+      </c>
+      <c r="ER2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="ES2" t="n">
+        <v>-0.151515</v>
+      </c>
+      <c r="ET2" t="n">
+        <v>-0.052525</v>
+      </c>
+      <c r="EU2" t="n">
+        <v>-0.098134</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>-0.203305</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>0.9408</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="EY2" t="n">
+        <v>69385</v>
+      </c>
+      <c r="EZ2" t="n">
+        <v>0.000385</v>
+      </c>
+      <c r="FA2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="GN2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="GO2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="GP2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="GQ2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="GR2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="GS2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="GT2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="GU2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="GV2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="GW2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="GX2" t="n">
+        <v>6</v>
+      </c>
+      <c r="GY2" t="inlineStr">
+        <is>
+          <t>Lego Corporate Finance Limited</t>
+        </is>
+      </c>
+      <c r="GZ2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="HA2" t="inlineStr">
+        <is>
+          <t>Combined offering: Public Offer (12,500,000 Shares) and Placing (112,500,000 Shares)</t>
+        </is>
+      </c>
+      <c r="HB2" t="n">
+        <v>4000</v>
       </c>
     </row>
   </sheetData>
@@ -2143,29 +2721,29 @@
     <col width="22" customWidth="1" min="132" max="132"/>
     <col width="22" customWidth="1" min="133" max="133"/>
     <col width="22" customWidth="1" min="134" max="134"/>
-    <col width="22" customWidth="1" min="135" max="135"/>
-    <col width="22" customWidth="1" min="136" max="136"/>
-    <col width="22" customWidth="1" min="137" max="137"/>
-    <col width="22" customWidth="1" min="138" max="138"/>
-    <col width="22" customWidth="1" min="139" max="139"/>
-    <col width="22" customWidth="1" min="140" max="140"/>
-    <col width="22" customWidth="1" min="141" max="141"/>
-    <col width="22" customWidth="1" min="142" max="142"/>
+    <col width="18" customWidth="1" min="135" max="135"/>
+    <col width="21" customWidth="1" min="136" max="136"/>
+    <col width="20" customWidth="1" min="137" max="137"/>
+    <col width="24" customWidth="1" min="138" max="138"/>
+    <col width="18" customWidth="1" min="139" max="139"/>
+    <col width="18" customWidth="1" min="140" max="140"/>
+    <col width="19" customWidth="1" min="141" max="141"/>
+    <col width="20" customWidth="1" min="142" max="142"/>
     <col width="22" customWidth="1" min="143" max="143"/>
-    <col width="22" customWidth="1" min="144" max="144"/>
-    <col width="22" customWidth="1" min="145" max="145"/>
-    <col width="22" customWidth="1" min="146" max="146"/>
-    <col width="22" customWidth="1" min="147" max="147"/>
-    <col width="22" customWidth="1" min="148" max="148"/>
-    <col width="22" customWidth="1" min="149" max="149"/>
-    <col width="22" customWidth="1" min="150" max="150"/>
+    <col width="21" customWidth="1" min="144" max="144"/>
+    <col width="20" customWidth="1" min="145" max="145"/>
+    <col width="24" customWidth="1" min="146" max="146"/>
+    <col width="18" customWidth="1" min="147" max="147"/>
+    <col width="18" customWidth="1" min="148" max="148"/>
+    <col width="19" customWidth="1" min="149" max="149"/>
+    <col width="20" customWidth="1" min="150" max="150"/>
     <col width="22" customWidth="1" min="151" max="151"/>
-    <col width="22" customWidth="1" min="152" max="152"/>
+    <col width="26" customWidth="1" min="152" max="152"/>
     <col width="22" customWidth="1" min="153" max="153"/>
-    <col width="22" customWidth="1" min="154" max="154"/>
+    <col width="24" customWidth="1" min="154" max="154"/>
     <col width="22" customWidth="1" min="155" max="155"/>
-    <col width="22" customWidth="1" min="156" max="156"/>
-    <col width="22" customWidth="1" min="157" max="157"/>
+    <col width="24" customWidth="1" min="156" max="156"/>
+    <col width="21" customWidth="1" min="157" max="157"/>
     <col width="22" customWidth="1" min="158" max="158"/>
     <col width="22" customWidth="1" min="159" max="159"/>
     <col width="22" customWidth="1" min="160" max="160"/>
@@ -2878,117 +3456,117 @@
           <t>Company Chinese Name</t>
         </is>
       </c>
-      <c r="EE1" s="30" t="inlineStr">
+      <c r="EE1" s="43" t="inlineStr">
         <is>
           <t>Current listing status</t>
         </is>
       </c>
-      <c r="EF1" s="30" t="inlineStr">
+      <c r="EF1" s="43" t="inlineStr">
         <is>
           <t>1-month post-IPO close price (HK$)</t>
         </is>
       </c>
-      <c r="EG1" s="30" t="inlineStr">
+      <c r="EG1" s="43" t="inlineStr">
         <is>
           <t>1-month BHR from Day-1 close (%)</t>
         </is>
       </c>
-      <c r="EH1" s="30" t="inlineStr">
+      <c r="EH1" s="43" t="inlineStr">
         <is>
           <t>1-month total return from offer price (%)</t>
         </is>
       </c>
-      <c r="EI1" s="30" t="inlineStr">
+      <c r="EI1" s="43" t="inlineStr">
         <is>
           <t>1-month HSI return (%)</t>
         </is>
       </c>
-      <c r="EJ1" s="30" t="inlineStr">
+      <c r="EJ1" s="43" t="inlineStr">
         <is>
           <t>1-month HSTECH return (%)</t>
         </is>
       </c>
-      <c r="EK1" s="30" t="inlineStr">
+      <c r="EK1" s="43" t="inlineStr">
         <is>
           <t>1-month wealth relative vs HSI</t>
         </is>
       </c>
-      <c r="EL1" s="30" t="inlineStr">
+      <c r="EL1" s="43" t="inlineStr">
         <is>
           <t>1-month wealth relative vs HSTECH</t>
         </is>
       </c>
-      <c r="EM1" s="30" t="inlineStr">
+      <c r="EM1" s="43" t="inlineStr">
         <is>
           <t>1-month average daily turnover (HK$)</t>
         </is>
       </c>
-      <c r="EN1" s="30" t="inlineStr">
+      <c r="EN1" s="43" t="inlineStr">
         <is>
           <t>6-month post-IPO close price (HK$)</t>
         </is>
       </c>
-      <c r="EO1" s="30" t="inlineStr">
+      <c r="EO1" s="43" t="inlineStr">
         <is>
           <t>6-month BHR from Day-1 close (%)</t>
         </is>
       </c>
-      <c r="EP1" s="30" t="inlineStr">
+      <c r="EP1" s="43" t="inlineStr">
         <is>
           <t>6-month total return from offer price (%)</t>
         </is>
       </c>
-      <c r="EQ1" s="30" t="inlineStr">
+      <c r="EQ1" s="43" t="inlineStr">
         <is>
           <t>6-month HSI return (%)</t>
         </is>
       </c>
-      <c r="ER1" s="30" t="inlineStr">
+      <c r="ER1" s="43" t="inlineStr">
         <is>
           <t>6-month HSTECH return (%)</t>
         </is>
       </c>
-      <c r="ES1" s="30" t="inlineStr">
+      <c r="ES1" s="43" t="inlineStr">
         <is>
           <t>6-month wealth relative vs HSI</t>
         </is>
       </c>
-      <c r="ET1" s="30" t="inlineStr">
+      <c r="ET1" s="43" t="inlineStr">
         <is>
           <t>6-month wealth relative vs HSTECH</t>
         </is>
       </c>
-      <c r="EU1" s="30" t="inlineStr">
+      <c r="EU1" s="43" t="inlineStr">
         <is>
           <t>6-month average daily turnover (HK$)</t>
         </is>
       </c>
-      <c r="EV1" s="30" t="inlineStr">
+      <c r="EV1" s="43" t="inlineStr">
         <is>
           <t>Liquidity decay ratio (6M vs Day-1 turnover)</t>
         </is>
       </c>
-      <c r="EW1" s="30" t="inlineStr">
+      <c r="EW1" s="43" t="inlineStr">
         <is>
           <t>1-year post-IPO return (%) [Reserved]</t>
         </is>
       </c>
-      <c r="EX1" s="30" t="inlineStr">
+      <c r="EX1" s="43" t="inlineStr">
         <is>
           <t>1-year wealth relative vs HSI [Reserved]</t>
         </is>
       </c>
-      <c r="EY1" s="30" t="inlineStr">
+      <c r="EY1" s="43" t="inlineStr">
         <is>
           <t>3-year post-IPO return (%) [Reserved]</t>
         </is>
       </c>
-      <c r="EZ1" s="30" t="inlineStr">
+      <c r="EZ1" s="43" t="inlineStr">
         <is>
           <t>3-year wealth relative vs HSI [Reserved]</t>
         </is>
       </c>
-      <c r="FA1" s="30" t="inlineStr">
+      <c r="FA1" s="43" t="inlineStr">
         <is>
           <t>18A/18C regulatory milestone status</t>
         </is>
@@ -3198,6 +3776,9 @@
           <t>BBSB International Limited</t>
         </is>
       </c>
+      <c r="D2" s="34" t="n">
+        <v>46022</v>
+      </c>
       <c r="E2" s="34" t="n">
         <v>46035</v>
       </c>
@@ -3213,6 +3794,472 @@
       </c>
       <c r="K2" t="n">
         <v>0.6</v>
+      </c>
+      <c r="L2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>375000000</v>
+      </c>
+      <c r="O2" t="n">
+        <v>375000000</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="R2" t="n">
+        <v>112500000</v>
+      </c>
+      <c r="S2" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="V2" s="49" t="n">
+        <v>-0.07692300000000001</v>
+      </c>
+      <c r="W2" s="49" t="n">
+        <v>0.153846</v>
+      </c>
+      <c r="X2" s="50" t="inlineStr">
+        <is>
+          <t>At low</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>MYR</t>
+        </is>
+      </c>
+      <c r="Z2" t="n">
+        <v>113572000</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>109044000</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>114046000</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>63611000</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>53800000</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>57001000</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>49961000</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>55244000</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>57045000</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>76757000</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>133002000</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>147972000</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>-13098000</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>33273000</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>11886000</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>-14460000</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>26189000</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>6402000</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Civil engineering contractor in Malaysia specialising in bridge engineering services as a subcontractor for large-scale transportation infrastructure engineering projects</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>Listing on GEM of the Stock Exchange by way of Share Offer (Public Offer and Placing)</t>
+        </is>
+      </c>
+      <c r="AW2" s="34" t="n">
+        <v>45838</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>-3480000</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>9086000</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>Family (Datuk Tan and spouse Datin Pan, via BBSB Overseas)</t>
+        </is>
+      </c>
+      <c r="BP2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>6042000</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>GEM</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>602030</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>HSICS (Hang Seng Industry Classification System) 2026</t>
+        </is>
+      </c>
+      <c r="BY2" s="34" t="n">
+        <v>45807</v>
+      </c>
+      <c r="BZ2" s="51" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>Cayman Islands</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>Petaling Jaya, Malaysia</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>IFRS Accounting Standards</t>
+        </is>
+      </c>
+      <c r="CE2" s="34" t="n">
+        <v>44927</v>
+      </c>
+      <c r="CF2" s="34" t="n">
+        <v>45291</v>
+      </c>
+      <c r="CG2" s="34" t="n">
+        <v>45292</v>
+      </c>
+      <c r="CH2" s="34" t="n">
+        <v>45657</v>
+      </c>
+      <c r="CI2" s="34" t="n">
+        <v>45658</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>73986000</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>5943000</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>3201000</v>
+      </c>
+      <c r="CM2" s="34" t="n">
+        <v>46022</v>
+      </c>
+      <c r="CN2" s="34" t="n">
+        <v>46030</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>15806000</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>113000</v>
+      </c>
+      <c r="CR2" t="inlineStr">
+        <is>
+          <t>Unqualified opinion</t>
+        </is>
+      </c>
+      <c r="CS2" t="n">
+        <v>25300000</v>
+      </c>
+      <c r="CT2" t="inlineStr">
+        <is>
+          <t>Mr. Choy Joo Seong; Mr. Tan Nam Joo</t>
+        </is>
+      </c>
+      <c r="CU2" t="n">
+        <v>0.186624</v>
+      </c>
+      <c r="CV2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CW2" t="n">
+        <v>10745.13</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>145089</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>134314148000</v>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>Subscription level 10,745.13 times</t>
+        </is>
+      </c>
+      <c r="DA2" s="34" t="n">
+        <v>46031</v>
+      </c>
+      <c r="DB2" s="34" t="n">
+        <v>46034</v>
+      </c>
+      <c r="DC2" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>112500000</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG2" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH2" t="inlineStr">
+        <is>
+          <t>No clawback: Claw-back triggered No; re-allocation procedure not applied; final Public Offer 12,500,000 and Placing 112,500,000 Shares</t>
+        </is>
+      </c>
+      <c r="DI2" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>0.2033</v>
+      </c>
+      <c r="DM2" t="inlineStr">
+        <is>
+          <t>Free float denominator = total issued shares upon listing (col_CZ); numerator = offer shares minus cornerstone allocation</t>
+        </is>
+      </c>
+      <c r="DN2" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="DO2" t="n">
+        <v>-0.00016594</v>
+      </c>
+      <c r="DP2" t="n">
+        <v>1</v>
+      </c>
+      <c r="DQ2" t="n">
+        <v>0.0321107</v>
+      </c>
+      <c r="DR2" t="n">
+        <v>53950000000</v>
+      </c>
+      <c r="DS2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="DT2" s="49" t="n">
+        <v>0.116667</v>
+      </c>
+      <c r="DU2" s="52" t="n">
+        <v>8750000</v>
+      </c>
+      <c r="DV2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DW2" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="DX2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="DY2" t="n">
+        <v>120963660</v>
+      </c>
+      <c r="DZ2" s="49" t="n">
+        <v>0.967709</v>
+      </c>
+      <c r="ED2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="EE2" s="44" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="EF2" s="45" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="EG2" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="EH2" s="46" t="n">
+        <v>0.116667</v>
+      </c>
+      <c r="EI2" s="46" t="n">
+        <v>0.006655</v>
+      </c>
+      <c r="EJ2" s="46" t="n">
+        <v>-0.07703699999999999</v>
+      </c>
+      <c r="EK2" s="47" t="n">
+        <v>0.9933999999999999</v>
+      </c>
+      <c r="EL2" s="47" t="n">
+        <v>1.0835</v>
+      </c>
+      <c r="EM2" s="48" t="n">
+        <v>11622003.5</v>
+      </c>
+      <c r="EN2" s="45" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="EO2" s="46" t="n">
+        <v>-0.151515</v>
+      </c>
+      <c r="EP2" s="46" t="n">
+        <v>-0.052525</v>
+      </c>
+      <c r="EQ2" s="46" t="n">
+        <v>-0.098134</v>
+      </c>
+      <c r="ER2" s="46" t="n">
+        <v>-0.203305</v>
+      </c>
+      <c r="ES2" s="47" t="n">
+        <v>0.9408</v>
+      </c>
+      <c r="ET2" s="47" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="EU2" s="48" t="n">
+        <v>69385</v>
+      </c>
+      <c r="EV2" s="46" t="n">
+        <v>0.000385</v>
+      </c>
+      <c r="EW2" s="46" t="n"/>
+      <c r="EX2" s="47" t="n"/>
+      <c r="EY2" s="46" t="n"/>
+      <c r="EZ2" s="47" t="n"/>
+      <c r="FA2" s="44" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3399,9 +4446,81 @@
           <t>BBSB International Limited</t>
         </is>
       </c>
+      <c r="D2" s="34" t="n">
+        <v>46022</v>
+      </c>
       <c r="E2" s="34" t="n">
         <v>46035</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Lego Corporate Finance Limited</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Combined offering: Public Offer (12,500,000 Shares) and Placing (112,500,000 Shares)</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>4000</v>
+      </c>
       <c r="U2" t="n">
         <v>75000000</v>
       </c>
@@ -3413,7 +4532,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>https://www2.hkexnews.hk/-/media/HKEXnews/Homepage/New-Listings/New-Listing-Information/New-Listing-Report/GEM/e_newlistings2026.xlsx</t>
+          <t>/Users/georgezhu/Desktop/UROP HK IPO/.claude/worktrees/code-review-repo-sync-008ff4/pipeline/sources/GEM/e_newlistings2026.xlsx</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>HKEX publication 31/12/2025 06:05; https://www1.hkexnews.hk/listedco/listconews/gem/2025/1231/2025123100007.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>